<commit_message>
updated main GSC export data
</commit_message>
<xml_diff>
--- a/gsc-export/Breadcrumbs.xlsx
+++ b/gsc-export/Breadcrumbs.xlsx
@@ -25,12 +25,6 @@
     <t>Valid</t>
   </si>
   <si>
-    <t>2025-11-23</t>
-  </si>
-  <si>
-    <t>2025-11-24</t>
-  </si>
-  <si>
     <t>2025-11-25</t>
   </si>
   <si>
@@ -287,6 +281,12 @@
   </si>
   <si>
     <t>2026-02-18</t>
+  </si>
+  <si>
+    <t>2026-02-19</t>
+  </si>
+  <si>
+    <t>2026-02-20</t>
   </si>
   <si>
     <t>Issue</t>
@@ -367,7 +367,7 @@
         <v>0.0</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>25.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="3">
@@ -378,7 +378,7 @@
         <v>0.0</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>25.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="4">
@@ -455,7 +455,7 @@
         <v>0.0</v>
       </c>
       <c r="C10" t="n" s="0">
-        <v>27.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="11">
@@ -466,7 +466,7 @@
         <v>0.0</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>27.0</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="12">
@@ -477,7 +477,7 @@
         <v>0.0</v>
       </c>
       <c r="C12" t="n" s="0">
-        <v>26.0</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="13">
@@ -499,7 +499,7 @@
         <v>0.0</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="15">
@@ -510,7 +510,7 @@
         <v>0.0</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="16">
@@ -521,7 +521,7 @@
         <v>0.0</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>26.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="17">
@@ -532,7 +532,7 @@
         <v>0.0</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>26.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="18">
@@ -543,7 +543,7 @@
         <v>0.0</v>
       </c>
       <c r="C18" t="n" s="0">
-        <v>27.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="19">
@@ -554,7 +554,7 @@
         <v>0.0</v>
       </c>
       <c r="C19" t="n" s="0">
-        <v>29.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="20">
@@ -565,7 +565,7 @@
         <v>0.0</v>
       </c>
       <c r="C20" t="n" s="0">
-        <v>29.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="21">
@@ -576,7 +576,7 @@
         <v>0.0</v>
       </c>
       <c r="C21" t="n" s="0">
-        <v>30.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="22">
@@ -587,7 +587,7 @@
         <v>0.0</v>
       </c>
       <c r="C22" t="n" s="0">
-        <v>30.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="23">
@@ -598,7 +598,7 @@
         <v>0.0</v>
       </c>
       <c r="C23" t="n" s="0">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="24">
@@ -620,7 +620,7 @@
         <v>0.0</v>
       </c>
       <c r="C25" t="n" s="0">
-        <v>32.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="26">
@@ -631,7 +631,7 @@
         <v>0.0</v>
       </c>
       <c r="C26" t="n" s="0">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="27">
@@ -642,7 +642,7 @@
         <v>0.0</v>
       </c>
       <c r="C27" t="n" s="0">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="28">
@@ -675,7 +675,7 @@
         <v>0.0</v>
       </c>
       <c r="C30" t="n" s="0">
-        <v>32.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="31">
@@ -686,7 +686,7 @@
         <v>0.0</v>
       </c>
       <c r="C31" t="n" s="0">
-        <v>32.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="32">
@@ -697,7 +697,7 @@
         <v>0.0</v>
       </c>
       <c r="C32" t="n" s="0">
-        <v>30.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="33">
@@ -708,7 +708,7 @@
         <v>0.0</v>
       </c>
       <c r="C33" t="n" s="0">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="34">
@@ -719,7 +719,7 @@
         <v>0.0</v>
       </c>
       <c r="C34" t="n" s="0">
-        <v>32.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="35">
@@ -730,7 +730,7 @@
         <v>0.0</v>
       </c>
       <c r="C35" t="n" s="0">
-        <v>32.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="36">
@@ -763,7 +763,7 @@
         <v>0.0</v>
       </c>
       <c r="C38" t="n" s="0">
-        <v>28.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="39">
@@ -774,7 +774,7 @@
         <v>0.0</v>
       </c>
       <c r="C39" t="n" s="0">
-        <v>28.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="40">
@@ -785,7 +785,7 @@
         <v>0.0</v>
       </c>
       <c r="C40" t="n" s="0">
-        <v>30.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="41">
@@ -796,7 +796,7 @@
         <v>0.0</v>
       </c>
       <c r="C41" t="n" s="0">
-        <v>29.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="42">
@@ -807,7 +807,7 @@
         <v>0.0</v>
       </c>
       <c r="C42" t="n" s="0">
-        <v>28.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="43">
@@ -818,7 +818,7 @@
         <v>0.0</v>
       </c>
       <c r="C43" t="n" s="0">
-        <v>28.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="44">
@@ -873,7 +873,7 @@
         <v>0.0</v>
       </c>
       <c r="C48" t="n" s="0">
-        <v>27.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="49">
@@ -884,7 +884,7 @@
         <v>0.0</v>
       </c>
       <c r="C49" t="n" s="0">
-        <v>27.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="50">
@@ -950,7 +950,7 @@
         <v>0.0</v>
       </c>
       <c r="C55" t="n" s="0">
-        <v>26.0</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="56">
@@ -961,7 +961,7 @@
         <v>0.0</v>
       </c>
       <c r="C56" t="n" s="0">
-        <v>26.0</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="57">
@@ -972,7 +972,7 @@
         <v>0.0</v>
       </c>
       <c r="C57" t="n" s="0">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="58">
@@ -994,7 +994,7 @@
         <v>0.0</v>
       </c>
       <c r="C59" t="n" s="0">
-        <v>26.0</v>
+        <v>24.0</v>
       </c>
     </row>
     <row r="60">
@@ -1005,7 +1005,7 @@
         <v>0.0</v>
       </c>
       <c r="C60" t="n" s="0">
-        <v>25.0</v>
+        <v>23.0</v>
       </c>
     </row>
     <row r="61">
@@ -1027,7 +1027,7 @@
         <v>0.0</v>
       </c>
       <c r="C62" t="n" s="0">
-        <v>23.0</v>
+        <v>24.0</v>
       </c>
     </row>
     <row r="63">
@@ -1049,7 +1049,7 @@
         <v>0.0</v>
       </c>
       <c r="C64" t="n" s="0">
-        <v>24.0</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="65">
@@ -1060,7 +1060,7 @@
         <v>0.0</v>
       </c>
       <c r="C65" t="n" s="0">
-        <v>24.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="66">
@@ -1071,7 +1071,7 @@
         <v>0.0</v>
       </c>
       <c r="C66" t="n" s="0">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="67">
@@ -1082,7 +1082,7 @@
         <v>0.0</v>
       </c>
       <c r="C67" t="n" s="0">
-        <v>26.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="68">
@@ -1093,7 +1093,7 @@
         <v>0.0</v>
       </c>
       <c r="C68" t="n" s="0">
-        <v>26.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="69">
@@ -1181,7 +1181,7 @@
         <v>0.0</v>
       </c>
       <c r="C76" t="n" s="0">
-        <v>28.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="77">
@@ -1203,7 +1203,7 @@
         <v>0.0</v>
       </c>
       <c r="C78" t="n" s="0">
-        <v>27.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="79">
@@ -1214,7 +1214,7 @@
         <v>0.0</v>
       </c>
       <c r="C79" t="n" s="0">
-        <v>28.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="80">
@@ -1225,7 +1225,7 @@
         <v>0.0</v>
       </c>
       <c r="C80" t="n" s="0">
-        <v>28.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="81">
@@ -1236,7 +1236,7 @@
         <v>0.0</v>
       </c>
       <c r="C81" t="n" s="0">
-        <v>29.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="82">
@@ -1258,7 +1258,7 @@
         <v>0.0</v>
       </c>
       <c r="C83" t="n" s="0">
-        <v>30.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="84">
@@ -1280,7 +1280,7 @@
         <v>0.0</v>
       </c>
       <c r="C85" t="n" s="0">
-        <v>31.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="86">
@@ -1324,7 +1324,7 @@
         <v>0.0</v>
       </c>
       <c r="C89" t="n" s="0">
-        <v>30.0</v>
+        <v>31.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated GSC export data
</commit_message>
<xml_diff>
--- a/gsc-export/Breadcrumbs.xlsx
+++ b/gsc-export/Breadcrumbs.xlsx
@@ -25,42 +25,6 @@
     <t>Valid</t>
   </si>
   <si>
-    <t>2026-02-18</t>
-  </si>
-  <si>
-    <t>2026-02-19</t>
-  </si>
-  <si>
-    <t>2026-02-20</t>
-  </si>
-  <si>
-    <t>2026-02-21</t>
-  </si>
-  <si>
-    <t>2026-02-22</t>
-  </si>
-  <si>
-    <t>2026-02-23</t>
-  </si>
-  <si>
-    <t>2026-02-24</t>
-  </si>
-  <si>
-    <t>2026-02-25</t>
-  </si>
-  <si>
-    <t>2026-02-26</t>
-  </si>
-  <si>
-    <t>2026-02-27</t>
-  </si>
-  <si>
-    <t>2026-02-28</t>
-  </si>
-  <si>
-    <t>2026-03-01</t>
-  </si>
-  <si>
     <t>2026-03-02</t>
   </si>
   <si>
@@ -293,6 +257,42 @@
   </si>
   <si>
     <t>2026-05-18</t>
+  </si>
+  <si>
+    <t>2026-05-19</t>
+  </si>
+  <si>
+    <t>2026-05-20</t>
+  </si>
+  <si>
+    <t>2026-05-21</t>
+  </si>
+  <si>
+    <t>2026-05-22</t>
+  </si>
+  <si>
+    <t>2026-05-23</t>
+  </si>
+  <si>
+    <t>2026-05-24</t>
+  </si>
+  <si>
+    <t>2026-05-25</t>
+  </si>
+  <si>
+    <t>2026-05-26</t>
+  </si>
+  <si>
+    <t>2026-05-27</t>
+  </si>
+  <si>
+    <t>2026-05-28</t>
+  </si>
+  <si>
+    <t>2026-05-29</t>
+  </si>
+  <si>
+    <t>2026-05-30</t>
   </si>
   <si>
     <t>Issue</t>
@@ -373,7 +373,7 @@
         <v>0.0</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>30.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="3">
@@ -384,7 +384,7 @@
         <v>0.0</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>30.0</v>
+        <v>34.0</v>
       </c>
     </row>
     <row r="4">
@@ -395,7 +395,7 @@
         <v>0.0</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>31.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="5">
@@ -406,7 +406,7 @@
         <v>0.0</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>31.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="6">
@@ -417,7 +417,7 @@
         <v>0.0</v>
       </c>
       <c r="C6" t="n" s="0">
-        <v>31.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="7">
@@ -428,7 +428,7 @@
         <v>0.0</v>
       </c>
       <c r="C7" t="n" s="0">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="8">
@@ -472,7 +472,7 @@
         <v>0.0</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>34.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="12">
@@ -483,7 +483,7 @@
         <v>0.0</v>
       </c>
       <c r="C12" t="n" s="0">
-        <v>34.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="13">
@@ -494,7 +494,7 @@
         <v>0.0</v>
       </c>
       <c r="C13" t="n" s="0">
-        <v>35.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="14">
@@ -505,7 +505,7 @@
         <v>0.0</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>35.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="15">
@@ -516,7 +516,7 @@
         <v>0.0</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>34.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="16">
@@ -527,7 +527,7 @@
         <v>0.0</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>35.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="17">
@@ -538,7 +538,7 @@
         <v>0.0</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>35.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="18">
@@ -549,7 +549,7 @@
         <v>0.0</v>
       </c>
       <c r="C18" t="n" s="0">
-        <v>35.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="19">
@@ -560,7 +560,7 @@
         <v>0.0</v>
       </c>
       <c r="C19" t="n" s="0">
-        <v>32.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="20">
@@ -571,7 +571,7 @@
         <v>0.0</v>
       </c>
       <c r="C20" t="n" s="0">
-        <v>32.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="21">
@@ -582,7 +582,7 @@
         <v>0.0</v>
       </c>
       <c r="C21" t="n" s="0">
-        <v>33.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="22">
@@ -593,7 +593,7 @@
         <v>0.0</v>
       </c>
       <c r="C22" t="n" s="0">
-        <v>33.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="23">
@@ -604,7 +604,7 @@
         <v>0.0</v>
       </c>
       <c r="C23" t="n" s="0">
-        <v>32.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="24">
@@ -615,7 +615,7 @@
         <v>0.0</v>
       </c>
       <c r="C24" t="n" s="0">
-        <v>32.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="25">
@@ -626,7 +626,7 @@
         <v>0.0</v>
       </c>
       <c r="C25" t="n" s="0">
-        <v>31.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="26">
@@ -637,7 +637,7 @@
         <v>0.0</v>
       </c>
       <c r="C26" t="n" s="0">
-        <v>31.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="27">
@@ -648,7 +648,7 @@
         <v>0.0</v>
       </c>
       <c r="C27" t="n" s="0">
-        <v>31.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="28">
@@ -659,7 +659,7 @@
         <v>0.0</v>
       </c>
       <c r="C28" t="n" s="0">
-        <v>28.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="29">
@@ -670,7 +670,7 @@
         <v>0.0</v>
       </c>
       <c r="C29" t="n" s="0">
-        <v>28.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="30">
@@ -692,7 +692,7 @@
         <v>0.0</v>
       </c>
       <c r="C31" t="n" s="0">
-        <v>29.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="32">
@@ -703,7 +703,7 @@
         <v>0.0</v>
       </c>
       <c r="C32" t="n" s="0">
-        <v>29.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="33">
@@ -714,7 +714,7 @@
         <v>0.0</v>
       </c>
       <c r="C33" t="n" s="0">
-        <v>29.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="34">
@@ -725,7 +725,7 @@
         <v>0.0</v>
       </c>
       <c r="C34" t="n" s="0">
-        <v>29.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="35">
@@ -736,7 +736,7 @@
         <v>0.0</v>
       </c>
       <c r="C35" t="n" s="0">
-        <v>29.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="36">
@@ -747,7 +747,7 @@
         <v>0.0</v>
       </c>
       <c r="C36" t="n" s="0">
-        <v>28.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="37">
@@ -758,7 +758,7 @@
         <v>0.0</v>
       </c>
       <c r="C37" t="n" s="0">
-        <v>28.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="38">
@@ -769,7 +769,7 @@
         <v>0.0</v>
       </c>
       <c r="C38" t="n" s="0">
-        <v>28.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="39">
@@ -780,7 +780,7 @@
         <v>0.0</v>
       </c>
       <c r="C39" t="n" s="0">
-        <v>28.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="40">
@@ -791,7 +791,7 @@
         <v>0.0</v>
       </c>
       <c r="C40" t="n" s="0">
-        <v>27.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="41">
@@ -802,7 +802,7 @@
         <v>0.0</v>
       </c>
       <c r="C41" t="n" s="0">
-        <v>29.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="42">
@@ -813,7 +813,7 @@
         <v>0.0</v>
       </c>
       <c r="C42" t="n" s="0">
-        <v>29.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="43">
@@ -824,7 +824,7 @@
         <v>0.0</v>
       </c>
       <c r="C43" t="n" s="0">
-        <v>30.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="44">
@@ -835,7 +835,7 @@
         <v>0.0</v>
       </c>
       <c r="C44" t="n" s="0">
-        <v>30.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="45">
@@ -846,7 +846,7 @@
         <v>0.0</v>
       </c>
       <c r="C45" t="n" s="0">
-        <v>30.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="46">
@@ -857,7 +857,7 @@
         <v>0.0</v>
       </c>
       <c r="C46" t="n" s="0">
-        <v>30.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="47">
@@ -868,7 +868,7 @@
         <v>0.0</v>
       </c>
       <c r="C47" t="n" s="0">
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="48">
@@ -890,7 +890,7 @@
         <v>0.0</v>
       </c>
       <c r="C49" t="n" s="0">
-        <v>31.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="50">
@@ -901,7 +901,7 @@
         <v>0.0</v>
       </c>
       <c r="C50" t="n" s="0">
-        <v>29.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="51">
@@ -912,7 +912,7 @@
         <v>0.0</v>
       </c>
       <c r="C51" t="n" s="0">
-        <v>29.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="52">
@@ -923,7 +923,7 @@
         <v>0.0</v>
       </c>
       <c r="C52" t="n" s="0">
-        <v>30.0</v>
+        <v>33.0</v>
       </c>
     </row>
     <row r="53">
@@ -934,7 +934,7 @@
         <v>0.0</v>
       </c>
       <c r="C53" t="n" s="0">
-        <v>31.0</v>
+        <v>33.0</v>
       </c>
     </row>
     <row r="54">
@@ -945,7 +945,7 @@
         <v>0.0</v>
       </c>
       <c r="C54" t="n" s="0">
-        <v>32.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="55">
@@ -956,7 +956,7 @@
         <v>0.0</v>
       </c>
       <c r="C55" t="n" s="0">
-        <v>32.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="56">
@@ -967,7 +967,7 @@
         <v>0.0</v>
       </c>
       <c r="C56" t="n" s="0">
-        <v>32.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="57">
@@ -978,7 +978,7 @@
         <v>0.0</v>
       </c>
       <c r="C57" t="n" s="0">
-        <v>32.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="58">
@@ -989,7 +989,7 @@
         <v>0.0</v>
       </c>
       <c r="C58" t="n" s="0">
-        <v>32.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="59">
@@ -1000,7 +1000,7 @@
         <v>0.0</v>
       </c>
       <c r="C59" t="n" s="0">
-        <v>32.0</v>
+        <v>34.0</v>
       </c>
     </row>
     <row r="60">
@@ -1011,7 +1011,7 @@
         <v>0.0</v>
       </c>
       <c r="C60" t="n" s="0">
-        <v>31.0</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="61">
@@ -1022,7 +1022,7 @@
         <v>0.0</v>
       </c>
       <c r="C61" t="n" s="0">
-        <v>30.0</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="62">
@@ -1033,7 +1033,7 @@
         <v>0.0</v>
       </c>
       <c r="C62" t="n" s="0">
-        <v>32.0</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="63">
@@ -1044,7 +1044,7 @@
         <v>0.0</v>
       </c>
       <c r="C63" t="n" s="0">
-        <v>32.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="64">
@@ -1055,7 +1055,7 @@
         <v>0.0</v>
       </c>
       <c r="C64" t="n" s="0">
-        <v>33.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="65">
@@ -1066,7 +1066,7 @@
         <v>0.0</v>
       </c>
       <c r="C65" t="n" s="0">
-        <v>33.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="66">
@@ -1077,7 +1077,7 @@
         <v>0.0</v>
       </c>
       <c r="C66" t="n" s="0">
-        <v>35.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="67">
@@ -1088,7 +1088,7 @@
         <v>0.0</v>
       </c>
       <c r="C67" t="n" s="0">
-        <v>35.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="68">
@@ -1099,7 +1099,7 @@
         <v>0.0</v>
       </c>
       <c r="C68" t="n" s="0">
-        <v>35.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="69">
@@ -1110,7 +1110,7 @@
         <v>0.0</v>
       </c>
       <c r="C69" t="n" s="0">
-        <v>35.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="70">
@@ -1121,7 +1121,7 @@
         <v>0.0</v>
       </c>
       <c r="C70" t="n" s="0">
-        <v>35.0</v>
+        <v>38.0</v>
       </c>
     </row>
     <row r="71">
@@ -1132,7 +1132,7 @@
         <v>0.0</v>
       </c>
       <c r="C71" t="n" s="0">
-        <v>34.0</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="72">
@@ -1143,7 +1143,7 @@
         <v>0.0</v>
       </c>
       <c r="C72" t="n" s="0">
-        <v>36.0</v>
+        <v>41.0</v>
       </c>
     </row>
     <row r="73">
@@ -1154,7 +1154,7 @@
         <v>0.0</v>
       </c>
       <c r="C73" t="n" s="0">
-        <v>36.0</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="74">
@@ -1165,7 +1165,7 @@
         <v>0.0</v>
       </c>
       <c r="C74" t="n" s="0">
-        <v>36.0</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="75">
@@ -1176,7 +1176,7 @@
         <v>0.0</v>
       </c>
       <c r="C75" t="n" s="0">
-        <v>37.0</v>
+        <v>42.0</v>
       </c>
     </row>
     <row r="76">
@@ -1187,7 +1187,7 @@
         <v>0.0</v>
       </c>
       <c r="C76" t="n" s="0">
-        <v>37.0</v>
+        <v>42.0</v>
       </c>
     </row>
     <row r="77">
@@ -1198,7 +1198,7 @@
         <v>0.0</v>
       </c>
       <c r="C77" t="n" s="0">
-        <v>37.0</v>
+        <v>43.0</v>
       </c>
     </row>
     <row r="78">
@@ -1209,7 +1209,7 @@
         <v>0.0</v>
       </c>
       <c r="C78" t="n" s="0">
-        <v>37.0</v>
+        <v>45.0</v>
       </c>
     </row>
     <row r="79">
@@ -1220,7 +1220,7 @@
         <v>0.0</v>
       </c>
       <c r="C79" t="n" s="0">
-        <v>37.0</v>
+        <v>45.0</v>
       </c>
     </row>
     <row r="80">
@@ -1231,7 +1231,7 @@
         <v>0.0</v>
       </c>
       <c r="C80" t="n" s="0">
-        <v>37.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="81">
@@ -1242,7 +1242,7 @@
         <v>0.0</v>
       </c>
       <c r="C81" t="n" s="0">
-        <v>37.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="82">
@@ -1253,7 +1253,7 @@
         <v>0.0</v>
       </c>
       <c r="C82" t="n" s="0">
-        <v>38.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="83">
@@ -1264,7 +1264,7 @@
         <v>0.0</v>
       </c>
       <c r="C83" t="n" s="0">
-        <v>40.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="84">
@@ -1275,7 +1275,7 @@
         <v>0.0</v>
       </c>
       <c r="C84" t="n" s="0">
-        <v>41.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="85">
@@ -1286,7 +1286,7 @@
         <v>0.0</v>
       </c>
       <c r="C85" t="n" s="0">
-        <v>40.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="86">
@@ -1297,7 +1297,7 @@
         <v>0.0</v>
       </c>
       <c r="C86" t="n" s="0">
-        <v>40.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="87">
@@ -1308,7 +1308,7 @@
         <v>0.0</v>
       </c>
       <c r="C87" t="n" s="0">
-        <v>42.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="88">
@@ -1319,7 +1319,7 @@
         <v>0.0</v>
       </c>
       <c r="C88" t="n" s="0">
-        <v>42.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="89">
@@ -1330,7 +1330,7 @@
         <v>0.0</v>
       </c>
       <c r="C89" t="n" s="0">
-        <v>43.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="90">
@@ -1341,7 +1341,7 @@
         <v>0.0</v>
       </c>
       <c r="C90" t="n" s="0">
-        <v>45.0</v>
+        <v>46.0</v>
       </c>
     </row>
     <row r="91">

</xml_diff>

<commit_message>
updated GSC index data
</commit_message>
<xml_diff>
--- a/gsc-export/Breadcrumbs.xlsx
+++ b/gsc-export/Breadcrumbs.xlsx
@@ -25,30 +25,6 @@
     <t>Valid</t>
   </si>
   <si>
-    <t>2026-04-12</t>
-  </si>
-  <si>
-    <t>2026-04-13</t>
-  </si>
-  <si>
-    <t>2026-04-14</t>
-  </si>
-  <si>
-    <t>2026-04-15</t>
-  </si>
-  <si>
-    <t>2026-04-16</t>
-  </si>
-  <si>
-    <t>2026-04-17</t>
-  </si>
-  <si>
-    <t>2026-04-18</t>
-  </si>
-  <si>
-    <t>2026-04-19</t>
-  </si>
-  <si>
     <t>2026-04-20</t>
   </si>
   <si>
@@ -293,6 +269,30 @@
   </si>
   <si>
     <t>2026-07-10</t>
+  </si>
+  <si>
+    <t>2026-07-11</t>
+  </si>
+  <si>
+    <t>2026-07-12</t>
+  </si>
+  <si>
+    <t>2026-07-13</t>
+  </si>
+  <si>
+    <t>2026-07-14</t>
+  </si>
+  <si>
+    <t>2026-07-15</t>
+  </si>
+  <si>
+    <t>2026-07-16</t>
+  </si>
+  <si>
+    <t>2026-07-17</t>
+  </si>
+  <si>
+    <t>2026-07-18</t>
   </si>
   <si>
     <t>Issue</t>
@@ -384,7 +384,7 @@
         <v>0.0</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>32.0</v>
+        <v>33.0</v>
       </c>
     </row>
     <row r="4">
@@ -395,7 +395,7 @@
         <v>0.0</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>32.0</v>
+        <v>33.0</v>
       </c>
     </row>
     <row r="5">
@@ -406,7 +406,7 @@
         <v>0.0</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>32.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="6">
@@ -417,7 +417,7 @@
         <v>0.0</v>
       </c>
       <c r="C6" t="n" s="0">
-        <v>32.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="7">
@@ -428,7 +428,7 @@
         <v>0.0</v>
       </c>
       <c r="C7" t="n" s="0">
-        <v>31.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="8">
@@ -439,7 +439,7 @@
         <v>0.0</v>
       </c>
       <c r="C8" t="n" s="0">
-        <v>30.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="9">
@@ -450,7 +450,7 @@
         <v>0.0</v>
       </c>
       <c r="C9" t="n" s="0">
-        <v>32.0</v>
+        <v>35.0</v>
       </c>
     </row>
     <row r="10">
@@ -461,7 +461,7 @@
         <v>0.0</v>
       </c>
       <c r="C10" t="n" s="0">
-        <v>32.0</v>
+        <v>34.0</v>
       </c>
     </row>
     <row r="11">
@@ -472,7 +472,7 @@
         <v>0.0</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>33.0</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="12">
@@ -483,7 +483,7 @@
         <v>0.0</v>
       </c>
       <c r="C12" t="n" s="0">
-        <v>33.0</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="13">
@@ -494,7 +494,7 @@
         <v>0.0</v>
       </c>
       <c r="C13" t="n" s="0">
-        <v>35.0</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="14">
@@ -505,7 +505,7 @@
         <v>0.0</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>35.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="15">
@@ -516,7 +516,7 @@
         <v>0.0</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>35.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="16">
@@ -527,7 +527,7 @@
         <v>0.0</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>35.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="17">
@@ -538,7 +538,7 @@
         <v>0.0</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>35.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="18">
@@ -549,7 +549,7 @@
         <v>0.0</v>
       </c>
       <c r="C18" t="n" s="0">
-        <v>34.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="19">
@@ -560,7 +560,7 @@
         <v>0.0</v>
       </c>
       <c r="C19" t="n" s="0">
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="20">
@@ -571,7 +571,7 @@
         <v>0.0</v>
       </c>
       <c r="C20" t="n" s="0">
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="21">
@@ -582,7 +582,7 @@
         <v>0.0</v>
       </c>
       <c r="C21" t="n" s="0">
-        <v>36.0</v>
+        <v>38.0</v>
       </c>
     </row>
     <row r="22">
@@ -593,7 +593,7 @@
         <v>0.0</v>
       </c>
       <c r="C22" t="n" s="0">
-        <v>37.0</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="23">
@@ -604,7 +604,7 @@
         <v>0.0</v>
       </c>
       <c r="C23" t="n" s="0">
-        <v>37.0</v>
+        <v>41.0</v>
       </c>
     </row>
     <row r="24">
@@ -615,7 +615,7 @@
         <v>0.0</v>
       </c>
       <c r="C24" t="n" s="0">
-        <v>37.0</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="25">
@@ -626,7 +626,7 @@
         <v>0.0</v>
       </c>
       <c r="C25" t="n" s="0">
-        <v>37.0</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="26">
@@ -637,7 +637,7 @@
         <v>0.0</v>
       </c>
       <c r="C26" t="n" s="0">
-        <v>37.0</v>
+        <v>42.0</v>
       </c>
     </row>
     <row r="27">
@@ -648,7 +648,7 @@
         <v>0.0</v>
       </c>
       <c r="C27" t="n" s="0">
-        <v>37.0</v>
+        <v>42.0</v>
       </c>
     </row>
     <row r="28">
@@ -659,7 +659,7 @@
         <v>0.0</v>
       </c>
       <c r="C28" t="n" s="0">
-        <v>37.0</v>
+        <v>43.0</v>
       </c>
     </row>
     <row r="29">
@@ -670,7 +670,7 @@
         <v>0.0</v>
       </c>
       <c r="C29" t="n" s="0">
-        <v>38.0</v>
+        <v>45.0</v>
       </c>
     </row>
     <row r="30">
@@ -681,7 +681,7 @@
         <v>0.0</v>
       </c>
       <c r="C30" t="n" s="0">
-        <v>40.0</v>
+        <v>45.0</v>
       </c>
     </row>
     <row r="31">
@@ -692,7 +692,7 @@
         <v>0.0</v>
       </c>
       <c r="C31" t="n" s="0">
-        <v>41.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="32">
@@ -703,7 +703,7 @@
         <v>0.0</v>
       </c>
       <c r="C32" t="n" s="0">
-        <v>40.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="33">
@@ -714,7 +714,7 @@
         <v>0.0</v>
       </c>
       <c r="C33" t="n" s="0">
-        <v>40.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="34">
@@ -725,7 +725,7 @@
         <v>0.0</v>
       </c>
       <c r="C34" t="n" s="0">
-        <v>42.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="35">
@@ -736,7 +736,7 @@
         <v>0.0</v>
       </c>
       <c r="C35" t="n" s="0">
-        <v>42.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="36">
@@ -747,7 +747,7 @@
         <v>0.0</v>
       </c>
       <c r="C36" t="n" s="0">
-        <v>43.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="37">
@@ -758,7 +758,7 @@
         <v>0.0</v>
       </c>
       <c r="C37" t="n" s="0">
-        <v>45.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="38">
@@ -769,7 +769,7 @@
         <v>0.0</v>
       </c>
       <c r="C38" t="n" s="0">
-        <v>45.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="39">
@@ -780,7 +780,7 @@
         <v>0.0</v>
       </c>
       <c r="C39" t="n" s="0">
-        <v>48.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="40">
@@ -791,7 +791,7 @@
         <v>0.0</v>
       </c>
       <c r="C40" t="n" s="0">
-        <v>48.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="41">
@@ -802,7 +802,7 @@
         <v>0.0</v>
       </c>
       <c r="C41" t="n" s="0">
-        <v>48.0</v>
+        <v>46.0</v>
       </c>
     </row>
     <row r="42">
@@ -813,7 +813,7 @@
         <v>0.0</v>
       </c>
       <c r="C42" t="n" s="0">
-        <v>48.0</v>
+        <v>45.0</v>
       </c>
     </row>
     <row r="43">
@@ -824,7 +824,7 @@
         <v>0.0</v>
       </c>
       <c r="C43" t="n" s="0">
-        <v>48.0</v>
+        <v>46.0</v>
       </c>
     </row>
     <row r="44">
@@ -835,7 +835,7 @@
         <v>0.0</v>
       </c>
       <c r="C44" t="n" s="0">
-        <v>48.0</v>
+        <v>46.0</v>
       </c>
     </row>
     <row r="45">
@@ -857,7 +857,7 @@
         <v>0.0</v>
       </c>
       <c r="C46" t="n" s="0">
-        <v>47.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="47">
@@ -868,7 +868,7 @@
         <v>0.0</v>
       </c>
       <c r="C47" t="n" s="0">
-        <v>47.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="48">
@@ -879,7 +879,7 @@
         <v>0.0</v>
       </c>
       <c r="C48" t="n" s="0">
-        <v>47.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="49">
@@ -890,7 +890,7 @@
         <v>0.0</v>
       </c>
       <c r="C49" t="n" s="0">
-        <v>46.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="50">
@@ -901,7 +901,7 @@
         <v>0.0</v>
       </c>
       <c r="C50" t="n" s="0">
-        <v>45.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="51">
@@ -912,7 +912,7 @@
         <v>0.0</v>
       </c>
       <c r="C51" t="n" s="0">
-        <v>46.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="52">
@@ -923,7 +923,7 @@
         <v>0.0</v>
       </c>
       <c r="C52" t="n" s="0">
-        <v>46.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="53">
@@ -934,7 +934,7 @@
         <v>0.0</v>
       </c>
       <c r="C53" t="n" s="0">
-        <v>48.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="54">
@@ -945,7 +945,7 @@
         <v>0.0</v>
       </c>
       <c r="C54" t="n" s="0">
-        <v>48.0</v>
+        <v>49.0</v>
       </c>
     </row>
     <row r="55">
@@ -956,7 +956,7 @@
         <v>0.0</v>
       </c>
       <c r="C55" t="n" s="0">
-        <v>48.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="56">
@@ -967,7 +967,7 @@
         <v>0.0</v>
       </c>
       <c r="C56" t="n" s="0">
-        <v>48.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="57">
@@ -978,7 +978,7 @@
         <v>0.0</v>
       </c>
       <c r="C57" t="n" s="0">
-        <v>48.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="58">
@@ -989,7 +989,7 @@
         <v>0.0</v>
       </c>
       <c r="C58" t="n" s="0">
-        <v>48.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="59">
@@ -1000,7 +1000,7 @@
         <v>0.0</v>
       </c>
       <c r="C59" t="n" s="0">
-        <v>48.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="60">
@@ -1011,7 +1011,7 @@
         <v>0.0</v>
       </c>
       <c r="C60" t="n" s="0">
-        <v>48.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="61">
@@ -1022,7 +1022,7 @@
         <v>0.0</v>
       </c>
       <c r="C61" t="n" s="0">
-        <v>47.0</v>
+        <v>56.0</v>
       </c>
     </row>
     <row r="62">
@@ -1033,7 +1033,7 @@
         <v>0.0</v>
       </c>
       <c r="C62" t="n" s="0">
-        <v>49.0</v>
+        <v>56.0</v>
       </c>
     </row>
     <row r="63">
@@ -1044,7 +1044,7 @@
         <v>0.0</v>
       </c>
       <c r="C63" t="n" s="0">
-        <v>52.0</v>
+        <v>56.0</v>
       </c>
     </row>
     <row r="64">
@@ -1055,7 +1055,7 @@
         <v>0.0</v>
       </c>
       <c r="C64" t="n" s="0">
-        <v>52.0</v>
+        <v>60.0</v>
       </c>
     </row>
     <row r="65">
@@ -1066,7 +1066,7 @@
         <v>0.0</v>
       </c>
       <c r="C65" t="n" s="0">
-        <v>52.0</v>
+        <v>62.0</v>
       </c>
     </row>
     <row r="66">
@@ -1077,7 +1077,7 @@
         <v>0.0</v>
       </c>
       <c r="C66" t="n" s="0">
-        <v>52.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="67">
@@ -1088,7 +1088,7 @@
         <v>0.0</v>
       </c>
       <c r="C67" t="n" s="0">
-        <v>54.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="68">
@@ -1099,7 +1099,7 @@
         <v>0.0</v>
       </c>
       <c r="C68" t="n" s="0">
-        <v>54.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="69">
@@ -1110,7 +1110,7 @@
         <v>0.0</v>
       </c>
       <c r="C69" t="n" s="0">
-        <v>56.0</v>
+        <v>63.0</v>
       </c>
     </row>
     <row r="70">
@@ -1121,7 +1121,7 @@
         <v>0.0</v>
       </c>
       <c r="C70" t="n" s="0">
-        <v>56.0</v>
+        <v>65.0</v>
       </c>
     </row>
     <row r="71">
@@ -1132,7 +1132,7 @@
         <v>0.0</v>
       </c>
       <c r="C71" t="n" s="0">
-        <v>56.0</v>
+        <v>65.0</v>
       </c>
     </row>
     <row r="72">
@@ -1143,7 +1143,7 @@
         <v>0.0</v>
       </c>
       <c r="C72" t="n" s="0">
-        <v>60.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="73">
@@ -1154,7 +1154,7 @@
         <v>0.0</v>
       </c>
       <c r="C73" t="n" s="0">
-        <v>62.0</v>
+        <v>65.0</v>
       </c>
     </row>
     <row r="74">
@@ -1198,7 +1198,7 @@
         <v>0.0</v>
       </c>
       <c r="C77" t="n" s="0">
-        <v>63.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="78">
@@ -1220,7 +1220,7 @@
         <v>0.0</v>
       </c>
       <c r="C79" t="n" s="0">
-        <v>65.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="80">
@@ -1242,7 +1242,7 @@
         <v>0.0</v>
       </c>
       <c r="C81" t="n" s="0">
-        <v>65.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="82">
@@ -1253,7 +1253,7 @@
         <v>0.0</v>
       </c>
       <c r="C82" t="n" s="0">
-        <v>64.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="83">
@@ -1264,7 +1264,7 @@
         <v>0.0</v>
       </c>
       <c r="C83" t="n" s="0">
-        <v>64.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="84">
@@ -1275,7 +1275,7 @@
         <v>0.0</v>
       </c>
       <c r="C84" t="n" s="0">
-        <v>64.0</v>
+        <v>68.0</v>
       </c>
     </row>
     <row r="85">
@@ -1286,7 +1286,7 @@
         <v>0.0</v>
       </c>
       <c r="C85" t="n" s="0">
-        <v>64.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="86">
@@ -1297,7 +1297,7 @@
         <v>0.0</v>
       </c>
       <c r="C86" t="n" s="0">
-        <v>65.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="87">
@@ -1308,7 +1308,7 @@
         <v>0.0</v>
       </c>
       <c r="C87" t="n" s="0">
-        <v>66.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="88">
@@ -1319,7 +1319,7 @@
         <v>0.0</v>
       </c>
       <c r="C88" t="n" s="0">
-        <v>66.0</v>
+        <v>68.0</v>
       </c>
     </row>
     <row r="89">
@@ -1330,7 +1330,7 @@
         <v>0.0</v>
       </c>
       <c r="C89" t="n" s="0">
-        <v>66.0</v>
+        <v>68.0</v>
       </c>
     </row>
     <row r="90">
@@ -1341,7 +1341,7 @@
         <v>0.0</v>
       </c>
       <c r="C90" t="n" s="0">
-        <v>67.0</v>
+        <v>69.0</v>
       </c>
     </row>
     <row r="91">
@@ -1352,7 +1352,7 @@
         <v>0.0</v>
       </c>
       <c r="C91" t="n" s="0">
-        <v>67.0</v>
+        <v>70.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>